<commit_message>
Deltavision fået status Godkendt for standarder.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF18831D87E345B446BBA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{536E7855-0BF0-4043-9AA3-D7D54751F7CF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8D33B1-F7CC-4229-A7E8-6FB2D67C7AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1632" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 14-09-2026" sheetId="1" r:id="rId1"/>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
opdatering for Vena psykolog
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8D33B1-F7CC-4229-A7E8-6FB2D67C7AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13DAF823-C597-4441-BB89-7B0C36B957F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="1632" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 14-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 17-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 14-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 17-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Opdateret XMedicus godkendte stausser
BIN01 (modtage) er vi godkendte i privath - vil I overføre det til SPL
RPT03 er vi godkendte til i LPS - vil I overføre dette til SPL
RPT04 er vi godkendte til  i LPS - vil I overføre dette til SPL
DIS13 er vi godkendte til i privath - vil i overføre dette til SPL
DIS91 er vi godkendte til i LPS og privath - vil I overføre til SPL
REF01 (modtage) er vi godkendte til - vil I overføre til SPL
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8725B7B8-1260-464B-BC44-11F8C5BF4DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF1883163B6F65B426ABA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70A6313A-7AC8-41B4-A181-9F7D4C5C41E1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 17-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 18-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 17-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 18-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Rettet fra ikke godkendt til godkendt jf. Pernille/XMedicus mail
"BIN01 (modtage) er vi godkendte i privath - vil I overføre det til SPL
RPT03 er vi godkendte til i LPS - vil I overføre dette til SPL
RPT04 er vi godkendte til  i LPS - vil I overføre dette til SPL
DIS13 er vi godkendte til i privath - vil i overføre dette til SPL
DIS91 er vi godkendte til i LPS og privath - vil I overføre til SPL
REF01 (modtage) er vi godkendte til - vil I overføre til SPL"
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF1883163B6F65B426ABA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70A6313A-7AC8-41B4-A181-9F7D4C5C41E1}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF188312F9EF74E1A6BBA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C9953CC-4ACF-4826-AE8B-56F1AE103635}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 18-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 21-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 18-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 21-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
opdateret EG Clinea med Godkendelse for CC v. 5.0
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF188312F9EF74E1A6BBA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C9953CC-4ACF-4826-AE8B-56F1AE103635}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1F6B44-C3CC-41E8-88AC-925715195F52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 21-09-2026" sheetId="1" r:id="rId1"/>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
opdateret - rettet fejl med "stanched"-bemærkning
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF6513A-795A-429E-BDBF-0E85B007DB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FF51EA-3EF3-4975-8E77-32D240D3A6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 22-09-2026" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
PraksisJournal oprettet og tilføjet FHIR standarder som tester
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FF51EA-3EF3-4975-8E77-32D240D3A6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C76E08C9-2E6A-41C1-82BF-2DF5CFCA8014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 22-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 23-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 22-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 23-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Rettet DIS07 til godkendt for XMedicus
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C76E08C9-2E6A-41C1-82BF-2DF5CFCA8014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF18831DAB6B169766ABA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EA3775C-05FF-42BD-B478-3E6A024C6584}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 23-09-2026" sheetId="1" r:id="rId1"/>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
xmo shared notes tilføjet
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF18831C136316D6C6BBA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC15C1CF-B864-45D5-AC80-685C3B03BAA4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A060515-40BC-483B-9CCA-82B597819F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="5410" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 24-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 28-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 24-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 28-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Opdateret status for Praksisjournal
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A060515-40BC-483B-9CCA-82B597819F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF18831495EB46FD46BBA520A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D950D96-7437-45AD-9DF0-133691EB1F59}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="5410" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 28-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 02-10-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 28-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 02-10-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Vena psykolog kvittering godkendt
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/ras_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33DD9981-8D75-416B-9F7C-A73312492EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_A52A79AB4805BBDBF18831CD6EB250D26BBA520E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3D07452-FC96-4586-8357-B08058227FC8}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 07-10-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 08-10-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 07-10-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 08-10-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
opdateret med Modulus sag
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D31938-3063-4D42-A9C5-D93498DF73A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114B68D1-1ED8-4E9D-B43B-1A29C917C43D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 09-10-2026" sheetId="1" r:id="rId1"/>

</xml_diff>